<commit_message>
implement login with differnt feature and reusable components functionality
</commit_message>
<xml_diff>
--- a/src/tests/test-data/TestSuite.xlsx
+++ b/src/tests/test-data/TestSuite.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QA\PLAYWRIGHT AUTOMATION\Playwright-framework-main\src\tests\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37D3FEF-F9C0-41B9-8B0E-E0037C501A1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6889005-5B05-4D2F-AD7B-BA3DF8BBE3A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="32">
   <si>
     <t>Seq_id</t>
   </si>
@@ -111,6 +111,24 @@
   </si>
   <si>
     <t>DV_1</t>
+  </si>
+  <si>
+    <t>User Should be Login TFS Application</t>
+  </si>
+  <si>
+    <t>Login TFS application with username and password</t>
+  </si>
+  <si>
+    <t>Login TFS Application</t>
+  </si>
+  <si>
+    <t>logout TFS Application</t>
+  </si>
+  <si>
+    <t>User should be logout TFS Application</t>
+  </si>
+  <si>
+    <t>Logout TFS Application</t>
   </si>
 </sst>
 </file>
@@ -727,16 +745,16 @@
         <v>11</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>9</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="H9" t="s">
         <v>25</v>
@@ -744,33 +762,80 @@
       <c r="I9" s="5"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="A10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
       <c r="I10" s="5"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
+      <c r="A11" s="5" t="s">
+        <v>18</v>
+      </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
+      <c r="D11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" t="s">
+        <v>17</v>
+      </c>
       <c r="I11" s="5"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
+      <c r="A12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
       <c r="I12" s="5"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -795,6 +860,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A1:H1 A5:H5 A4 C4:H4 A3:G3 A7:H8 A6 C6:H6 A2 C2:H2" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>